<commit_message>
Update Iteracion 2 notes in test matrix
</commit_message>
<xml_diff>
--- a/docs/MRP_Piedrazul_v1.xlsx
+++ b/docs/MRP_Piedrazul_v1.xlsx
@@ -1350,11 +1350,19 @@
       </c>
       <c r="O10" s="44" t="inlineStr">
         <is>
-          <t>PDTE</t>
-        </is>
-      </c>
-      <c r="P10" s="45" t="n"/>
-      <c r="Q10" s="45" t="n"/>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="P10" s="45" t="inlineStr">
+        <is>
+          <t>Se cambia respuesta a 409 cuando el slot esta ocupado.</t>
+        </is>
+      </c>
+      <c r="Q10" s="45" t="inlineStr">
+        <is>
+          <t>Juan Felipe Ramirez</t>
+        </is>
+      </c>
       <c r="R10" s="44" t="inlineStr">
         <is>
           <t>PDTE</t>
@@ -1432,11 +1440,19 @@
       </c>
       <c r="O11" s="44" t="inlineStr">
         <is>
-          <t>PDTE</t>
-        </is>
-      </c>
-      <c r="P11" s="42" t="n"/>
-      <c r="Q11" s="42" t="n"/>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="P11" s="42" t="inlineStr">
+        <is>
+          <t>ModelState ahora retorna 422 con errors.</t>
+        </is>
+      </c>
+      <c r="Q11" s="42" t="inlineStr">
+        <is>
+          <t>Juan Felipe Ramirez</t>
+        </is>
+      </c>
       <c r="R11" s="44" t="inlineStr">
         <is>
           <t>PDTE</t>
@@ -2760,11 +2776,19 @@
       </c>
       <c r="O27" s="44" t="inlineStr">
         <is>
-          <t>PDTE</t>
-        </is>
-      </c>
-      <c r="P27" s="42" t="n"/>
-      <c r="Q27" s="42" t="n"/>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="P27" s="42" t="inlineStr">
+        <is>
+          <t>Cancelacion de cita ajena retorna 404.</t>
+        </is>
+      </c>
+      <c r="Q27" s="42" t="inlineStr">
+        <is>
+          <t>Juan Felipe Ramirez</t>
+        </is>
+      </c>
       <c r="R27" s="44" t="inlineStr">
         <is>
           <t>PDTE</t>
@@ -3658,11 +3682,19 @@
       </c>
       <c r="O38" s="44" t="inlineStr">
         <is>
-          <t>PDTE</t>
-        </is>
-      </c>
-      <c r="P38" s="45" t="n"/>
-      <c r="Q38" s="45" t="n"/>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="P38" s="45" t="inlineStr">
+        <is>
+          <t>Exportacion sin citas retorna 404.</t>
+        </is>
+      </c>
+      <c r="Q38" s="45" t="inlineStr">
+        <is>
+          <t>Juan Felipe Ramirez</t>
+        </is>
+      </c>
       <c r="R38" s="44" t="inlineStr">
         <is>
           <t>PDTE</t>
@@ -4314,11 +4346,19 @@
       </c>
       <c r="O46" s="44" t="inlineStr">
         <is>
-          <t>PDTE</t>
-        </is>
-      </c>
-      <c r="P46" s="45" t="n"/>
-      <c r="Q46" s="45" t="n"/>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="P46" s="45" t="inlineStr">
+        <is>
+          <t>Proveedor inactivo ya no aparece en listados.</t>
+        </is>
+      </c>
+      <c r="Q46" s="45" t="inlineStr">
+        <is>
+          <t>Juan Felipe Ramirez</t>
+        </is>
+      </c>
       <c r="R46" s="44" t="inlineStr">
         <is>
           <t>PDTE</t>
@@ -4628,7 +4668,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="24" customHeight="1" s="35">
       <c r="A3" s="50" t="inlineStr">
         <is>
@@ -5661,7 +5700,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="21.75" customHeight="1" s="35">
       <c r="A6" s="40" t="inlineStr">
         <is>
@@ -5797,7 +5835,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="21.75" customHeight="1" s="35">
       <c r="A10" s="40" t="inlineStr">
         <is>
@@ -5933,8 +5970,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15" ht="18" customHeight="1" s="35">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -5978,7 +6013,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="57" t="inlineStr">
         <is>
@@ -6027,7 +6061,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="35">
       <c r="A8" s="59" t="inlineStr">
         <is>
@@ -6095,7 +6128,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="35">
       <c r="A15" s="59" t="inlineStr">
         <is>
@@ -6171,7 +6203,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="35">
       <c r="A21" s="59" t="inlineStr">
         <is>
@@ -6378,7 +6409,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="31.5" customHeight="1" s="35">
       <c r="A3" s="41" t="inlineStr">
         <is>
@@ -9186,166 +9216,166 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>Resumen validacion (1a iteracion)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="34" t="inlineStr">
         <is>
           <t>Ejecuta</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="34" t="inlineStr">
         <is>
           <t>Juan Felipe Ramirez</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="34" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="34" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>Casos totales</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="34" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="34" t="inlineStr">
         <is>
           <t>Ejecutados</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="34" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="34" t="inlineStr">
         <is>
           <t>ENA</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="34" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>PDTE</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>PDTE</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="34" t="inlineStr">
         <is>
           <t>Correctitud</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="34" t="n">
         <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="34" t="inlineStr">
         <is>
           <t>Confiabilidad</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="34" t="n">
         <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="34" t="inlineStr">
         <is>
           <t>ENA (casos)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="34" t="inlineStr">
         <is>
           <t>PUB-06</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="34" t="inlineStr">
         <is>
           <t>Reserva en slot ocupado responde 400 (esperado 409).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>PUB-07</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>Validacion responde 400 (esperado 422).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="34" t="inlineStr">
         <is>
           <t>PAC-06</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>Cancelacion de cita ajena responde 400 (esperado 403/404).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t>INT-11</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>PDF sin citas responde 200 con archivo vacio (esperado 404).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="34" t="inlineStr">
         <is>
           <t>ADM-07</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="34" t="inlineStr">
         <is>
           <t>Proveedor permanece en listado; solo se elimina disponibilidad semanal.</t>
         </is>

</xml_diff>